<commit_message>
P1-T01: Scaffold Next.js 16 + Tailwind 4 + shadcn/ui
- Next.js App Router, TypeScript strict, ESLint, src/ layout
- Exact-pinned dependencies (.npmrc save-exact) with lockfile
- shadcn/ui initialised (base-nova style)
- .env.example with placeholders only
- LinkUp placeholder home page and metadata
- Tracker: P1-T01 Done, stack decision recorded

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project_tracker.xlsx
+++ b/docs/project_tracker.xlsx
@@ -20,8 +20,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$N$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Security'!$A$1:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Risks'!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions'!$A$1:$D$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Changelog'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Changelog'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -519,6 +519,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1011,7 +1012,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -1036,10 +1037,13 @@
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>create-next-app refuses non-empty dirs: scaffold into a temp folder and move files in (keep existing .gitignore, docs/, scripts/, CLAUDE.md).</t>
-        </is>
-      </c>
-      <c r="N2" s="8" t="n"/>
+          <t>create-next-app refuses non-empty dirs: scaffold into a temp folder and move files in (keep existing .gitignore, docs/, scripts/, CLAUDE.md).
+[2026-09-25] Next 16.3.6 scaffolded; exact-pinned deps; lint+build pass; dev serves 200; .env.local ignored; npm audit 0 vulns</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="n">
+        <v>46290</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -3950,7 +3954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4181,8 +4185,28 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Stack versions: Next.js 16.3.6, React 19.2, Tailwind 4, shadcn/ui 'base-nova' style (Base UI primitives, 'cn' package)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>shadcn Radix-based styles</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>create-next-app/shadcn defaults at scaffold time; Next 16 uses proxy.ts instead of middleware.ts; read node_modules/next/dist/docs before using unfamiliar APIs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D11"/>
+  <autoFilter ref="A1:D12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4193,7 +4217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4233,8 +4257,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Decision recorded: Stack versions: Next.js 16.3.6, React 19.2, Tailwind 4, shadcn/ui 'base-nova' style (Base UI primitives, 'cn' package)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>P1-T01</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Marked Done: Next 16.3.6 scaffolded; exact-pinned deps; lint+build pass; dev serves 200; .env.local ignored; npm audit 0 vulns</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:C4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>